<commit_message>
functioning weekly and joined streamlit app
</commit_message>
<xml_diff>
--- a/ΕΝΗΜΕΡΩΤΙΚΑ_ΣΗΜΕΙΩΜΑΤΑ/2026-02/XLSX/ΕΝΗΜΕΡΩΤΙΚΟ_ΣΗΜΕΙΩΜΑ_ΕΝΕΡΓΕΙΑΚΗ_ΚΟΙΝΟΤΗΤΑ_ΗΛΙΑΧΤΙΔΑ_Π.Ε._-_ΜΑΡΜΑΡΑ_2026-02.xlsx
+++ b/ΕΝΗΜΕΡΩΤΙΚΑ_ΣΗΜΕΙΩΜΑΤΑ/2026-02/XLSX/ΕΝΗΜΕΡΩΤΙΚΟ_ΣΗΜΕΙΩΜΑ_ΕΝΕΡΓΕΙΑΚΗ_ΚΟΙΝΟΤΗΤΑ_ΗΛΙΑΧΤΙΔΑ_Π.Ε._-_ΜΑΡΜΑΡΑ_2026-02.xlsx
@@ -2844,7 +2844,7 @@
     <row r="6" ht="60.75" customFormat="1" customHeight="1" s="10">
       <c r="B6" s="80" t="inlineStr">
         <is>
-          <t>09/03/26</t>
+          <t>03/04/26</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="C53" s="110" t="inlineStr">
         <is>
-          <t>11/03/26</t>
+          <t>05/04/26</t>
         </is>
       </c>
       <c r="D53" s="111" t="n"/>

</xml_diff>